<commit_message>
1 okt. 2026 v1
</commit_message>
<xml_diff>
--- a/filer_1/10360641_jem_fix_a_s.xlsx
+++ b/filer_1/10360641_jem_fix_a_s.xlsx
@@ -5083,11 +5083,21 @@
           <t>Finansielle poster, netto</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
+      <c r="B15" s="17" t="n">
+        <v>12721</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>-27449</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>56914</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>58270</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>62952</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">

</xml_diff>